<commit_message>
merenje halucinacije i korekcija chatrova
</commit_message>
<xml_diff>
--- a/dataset_evaluacija_llm_sa_odgovorima.xlsx
+++ b/dataset_evaluacija_llm_sa_odgovorima.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cofi24\Desktop\Git uploads\Evaluacija-jezickih-modela\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6C7BECD-A76A-42A7-9F5F-DC246CA27332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEBD384E-8492-4504-BE3A-C94764573722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tačnost" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1664" uniqueCount="1041">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1786" uniqueCount="1041">
   <si>
     <t>EVALUACIJA LLM-OVA NA SRPSKOM — KONZISTENTNOST</t>
   </si>
@@ -3959,21 +3959,12 @@
     <t>Konzistentnost: Consistency rate = (iste grupe / ukupno grupa) × 100%</t>
   </si>
   <si>
-    <t>Ne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ne </t>
-  </si>
-  <si>
     <t>Tačno_GPT (DA/NE)</t>
   </si>
   <si>
     <t>Tačno_Claude (DA/NE)</t>
   </si>
   <si>
-    <t>Tačno_Mistral  (DA/NE)</t>
-  </si>
-  <si>
     <t>Da li je halucinirao Mistral? (DA/NE)</t>
   </si>
   <si>
@@ -3996,6 +3987,15 @@
   </si>
   <si>
     <t>Nema najzdravije hrane ni pod kojim kriterijumima</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DA  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> NE</t>
+  </si>
+  <si>
+    <t>Tačno_Mistral (DA/NE)</t>
   </si>
 </sst>
 </file>
@@ -4619,13 +4619,13 @@
         <v>8</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>1030</v>
+        <v>1028</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>1031</v>
+        <v>1029</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>1032</v>
+        <v>1040</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>12</v>
@@ -4663,13 +4663,13 @@
         <v>139</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
@@ -4703,13 +4703,13 @@
         <v>146</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M4" s="5"/>
       <c r="N4" s="5"/>
@@ -4743,13 +4743,13 @@
         <v>152</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M5" s="3"/>
       <c r="N5" s="3"/>
@@ -4783,18 +4783,18 @@
         <v>158</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M6" s="5"/>
       <c r="N6" s="5"/>
     </row>
-    <row r="7" spans="1:14" ht="267.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" ht="255" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>160</v>
       </c>
@@ -4823,13 +4823,13 @@
         <v>165</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M7" s="3"/>
       <c r="N7" s="3"/>
@@ -4863,18 +4863,18 @@
         <v>170</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L8" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M8" s="5"/>
       <c r="N8" s="5"/>
     </row>
-    <row r="9" spans="1:14" ht="216.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="191.25" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>172</v>
       </c>
@@ -4903,13 +4903,13 @@
         <v>179</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M9" s="3"/>
       <c r="N9" s="3"/>
@@ -4943,13 +4943,13 @@
         <v>184</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L10" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M10" s="5"/>
       <c r="N10" s="5"/>
@@ -4983,13 +4983,13 @@
         <v>100</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M11" s="3"/>
       <c r="N11" s="3"/>
@@ -5023,13 +5023,13 @@
         <v>195</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L12" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M12" s="5"/>
       <c r="N12" s="5"/>
@@ -5063,13 +5063,13 @@
         <v>202</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M13" s="3"/>
       <c r="N13" s="3"/>
@@ -5103,13 +5103,13 @@
         <v>208</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L14" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M14" s="5"/>
       <c r="N14" s="5"/>
@@ -5143,13 +5143,13 @@
         <v>214</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M15" s="3"/>
       <c r="N15" s="3"/>
@@ -5183,18 +5183,18 @@
         <v>221</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L16" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M16" s="5"/>
       <c r="N16" s="5"/>
     </row>
-    <row r="17" spans="1:14" ht="267.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" ht="255" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>222</v>
       </c>
@@ -5205,7 +5205,7 @@
         <v>223</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>1038</v>
+        <v>1035</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>224</v>
@@ -5223,18 +5223,18 @@
         <v>227</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M17" s="3"/>
       <c r="N17" s="3"/>
     </row>
-    <row r="18" spans="1:14" ht="216.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" ht="191.25" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>228</v>
       </c>
@@ -5263,18 +5263,18 @@
         <v>235</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="L18" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M18" s="5"/>
       <c r="N18" s="5"/>
     </row>
-    <row r="19" spans="1:14" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" ht="140.25" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>236</v>
       </c>
@@ -5303,13 +5303,13 @@
         <v>241</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M19" s="3"/>
       <c r="N19" s="3"/>
@@ -5343,13 +5343,13 @@
         <v>249</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L20" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M20" s="5"/>
       <c r="N20" s="5"/>
@@ -5383,13 +5383,13 @@
         <v>256</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M21" s="3"/>
       <c r="N21" s="3"/>
@@ -5423,13 +5423,13 @@
         <v>263</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L22" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M22" s="5"/>
       <c r="N22" s="5"/>
@@ -5463,13 +5463,13 @@
         <v>271</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M23" s="3"/>
       <c r="N23" s="3"/>
@@ -5503,13 +5503,13 @@
         <v>277</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L24" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M24" s="5"/>
       <c r="N24" s="5"/>
@@ -5543,13 +5543,13 @@
         <v>285</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M25" s="3"/>
       <c r="N25" s="3"/>
@@ -5568,7 +5568,7 @@
         <v>289</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>1039</v>
+        <v>1036</v>
       </c>
       <c r="F26" s="23" t="s">
         <v>15</v>
@@ -5583,13 +5583,13 @@
         <v>292</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L26" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M26" s="5"/>
       <c r="N26" s="5"/>
@@ -5623,13 +5623,13 @@
         <v>300</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M27" s="3"/>
       <c r="N27" s="3"/>
@@ -5663,13 +5663,13 @@
         <v>307</v>
       </c>
       <c r="J28" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L28" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M28" s="5"/>
       <c r="N28" s="5"/>
@@ -5703,13 +5703,13 @@
         <v>313</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L29" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M29" s="3"/>
       <c r="N29" s="3"/>
@@ -5743,13 +5743,13 @@
         <v>320</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="L30" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M30" s="5"/>
       <c r="N30" s="5"/>
@@ -5781,13 +5781,13 @@
         <v>327</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K31" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L31" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M31" s="3"/>
       <c r="N31" s="3"/>
@@ -5821,13 +5821,13 @@
         <v>334</v>
       </c>
       <c r="J32" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L32" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M32" s="5"/>
       <c r="N32" s="5"/>
@@ -5861,13 +5861,13 @@
         <v>341</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K33" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M33" s="3"/>
       <c r="N33" s="3"/>
@@ -5901,13 +5901,13 @@
         <v>348</v>
       </c>
       <c r="J34" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L34" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M34" s="5"/>
       <c r="N34" s="5"/>
@@ -5941,18 +5941,18 @@
         <v>354</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="K35" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L35" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M35" s="3"/>
       <c r="N35" s="3"/>
     </row>
-    <row r="36" spans="1:14" ht="408" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" ht="395.25" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
         <v>355</v>
       </c>
@@ -5981,13 +5981,13 @@
         <v>362</v>
       </c>
       <c r="J36" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L36" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M36" s="5"/>
       <c r="N36" s="5"/>
@@ -6021,13 +6021,13 @@
         <v>368</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L37" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M37" s="3"/>
       <c r="N37" s="3"/>
@@ -6061,13 +6061,13 @@
         <v>375</v>
       </c>
       <c r="J38" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L38" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M38" s="5"/>
       <c r="N38" s="5"/>
@@ -6101,13 +6101,13 @@
         <v>382</v>
       </c>
       <c r="J39" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K39" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L39" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M39" s="3"/>
       <c r="N39" s="3"/>
@@ -6141,13 +6141,13 @@
         <v>389</v>
       </c>
       <c r="J40" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K40" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L40" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M40" s="5"/>
       <c r="N40" s="5"/>
@@ -6163,7 +6163,7 @@
         <v>391</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>1040</v>
+        <v>1037</v>
       </c>
       <c r="E41" s="21" t="s">
         <v>317</v>
@@ -6181,13 +6181,13 @@
         <v>394</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K41" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="L41" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M41" s="3"/>
       <c r="N41" s="3"/>
@@ -6221,13 +6221,13 @@
         <v>400</v>
       </c>
       <c r="J42" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K42" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L42" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M42" s="5"/>
       <c r="N42" s="5"/>
@@ -6261,13 +6261,13 @@
         <v>406</v>
       </c>
       <c r="J43" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K43" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L43" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M43" s="3"/>
       <c r="N43" s="3"/>
@@ -6301,13 +6301,13 @@
         <v>413</v>
       </c>
       <c r="J44" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K44" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L44" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M44" s="5"/>
       <c r="N44" s="5"/>
@@ -6341,13 +6341,13 @@
         <v>420</v>
       </c>
       <c r="J45" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K45" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L45" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M45" s="3"/>
       <c r="N45" s="3"/>
@@ -6381,13 +6381,13 @@
         <v>427</v>
       </c>
       <c r="J46" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K46" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="L46" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M46" s="5"/>
       <c r="N46" s="5"/>
@@ -6421,13 +6421,13 @@
         <v>434</v>
       </c>
       <c r="J47" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K47" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L47" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M47" s="3"/>
       <c r="N47" s="3"/>
@@ -6461,18 +6461,18 @@
         <v>442</v>
       </c>
       <c r="J48" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K48" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="L48" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M48" s="5"/>
       <c r="N48" s="5"/>
     </row>
-    <row r="49" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>443</v>
       </c>
@@ -6501,13 +6501,13 @@
         <v>449</v>
       </c>
       <c r="J49" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K49" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L49" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M49" s="3"/>
       <c r="N49" s="3"/>
@@ -6541,13 +6541,13 @@
         <v>457</v>
       </c>
       <c r="J50" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K50" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="L50" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M50" s="5"/>
       <c r="N50" s="5"/>
@@ -6581,13 +6581,13 @@
         <v>464</v>
       </c>
       <c r="J51" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K51" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="L51" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M51" s="3"/>
       <c r="N51" s="3"/>
@@ -6621,13 +6621,13 @@
         <v>470</v>
       </c>
       <c r="J52" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K52" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L52" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M52" s="5"/>
       <c r="N52" s="5"/>
@@ -6661,18 +6661,18 @@
         <v>477</v>
       </c>
       <c r="J53" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K53" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L53" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M53" s="3"/>
       <c r="N53" s="3"/>
     </row>
-    <row r="54" spans="1:14" ht="318.75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14" ht="306" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
         <v>478</v>
       </c>
@@ -6701,13 +6701,13 @@
         <v>483</v>
       </c>
       <c r="J54" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K54" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L54" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M54" s="5"/>
       <c r="N54" s="5"/>
@@ -6741,18 +6741,18 @@
         <v>490</v>
       </c>
       <c r="J55" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="K55" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="L55" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M55" s="3"/>
       <c r="N55" s="3"/>
     </row>
-    <row r="56" spans="1:14" ht="408" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" ht="382.5" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
         <v>491</v>
       </c>
@@ -6781,13 +6781,13 @@
         <v>497</v>
       </c>
       <c r="J56" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K56" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L56" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M56" s="5"/>
       <c r="N56" s="5"/>
@@ -6821,13 +6821,13 @@
         <v>503</v>
       </c>
       <c r="J57" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K57" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L57" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M57" s="3"/>
       <c r="N57" s="3"/>
@@ -6861,13 +6861,13 @@
         <v>509</v>
       </c>
       <c r="J58" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K58" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L58" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M58" s="5"/>
       <c r="N58" s="5"/>
@@ -6901,13 +6901,13 @@
         <v>516</v>
       </c>
       <c r="J59" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K59" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L59" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M59" s="3"/>
       <c r="N59" s="3"/>
@@ -6941,13 +6941,13 @@
         <v>523</v>
       </c>
       <c r="J60" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="K60" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L60" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M60" s="5"/>
       <c r="N60" s="5"/>
@@ -6981,13 +6981,13 @@
         <v>529</v>
       </c>
       <c r="J61" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K61" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L61" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M61" s="3"/>
       <c r="N61" s="3"/>
@@ -7021,13 +7021,13 @@
         <v>536</v>
       </c>
       <c r="J62" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K62" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L62" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M62" s="5"/>
       <c r="N62" s="5"/>
@@ -7061,13 +7061,13 @@
         <v>542</v>
       </c>
       <c r="J63" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K63" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L63" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M63" s="3"/>
       <c r="N63" s="3"/>
@@ -7101,13 +7101,13 @@
         <v>550</v>
       </c>
       <c r="J64" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K64" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L64" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M64" s="5"/>
       <c r="N64" s="5"/>
@@ -7141,13 +7141,13 @@
         <v>557</v>
       </c>
       <c r="J65" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K65" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L65" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M65" s="3"/>
       <c r="N65" s="3"/>
@@ -7181,13 +7181,13 @@
         <v>563</v>
       </c>
       <c r="J66" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K66" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L66" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M66" s="5"/>
       <c r="N66" s="5"/>
@@ -7221,13 +7221,13 @@
         <v>570</v>
       </c>
       <c r="J67" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K67" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L67" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M67" s="3"/>
       <c r="N67" s="3"/>
@@ -7261,13 +7261,13 @@
         <v>577</v>
       </c>
       <c r="J68" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="K68" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="L68" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M68" s="5"/>
       <c r="N68" s="5"/>
@@ -7301,13 +7301,13 @@
         <v>584</v>
       </c>
       <c r="J69" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K69" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L69" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M69" s="3"/>
       <c r="N69" s="3"/>
@@ -7341,13 +7341,13 @@
         <v>590</v>
       </c>
       <c r="J70" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K70" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L70" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M70" s="5"/>
       <c r="N70" s="5"/>
@@ -7381,13 +7381,13 @@
         <v>597</v>
       </c>
       <c r="J71" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K71" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L71" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M71" s="3"/>
       <c r="N71" s="3"/>
@@ -7421,13 +7421,13 @@
         <v>604</v>
       </c>
       <c r="J72" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K72" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L72" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M72" s="5"/>
       <c r="N72" s="5"/>
@@ -7461,13 +7461,13 @@
         <v>610</v>
       </c>
       <c r="J73" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="K73" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="L73" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M73" s="3"/>
       <c r="N73" s="3"/>
@@ -7501,13 +7501,13 @@
         <v>617</v>
       </c>
       <c r="J74" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K74" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L74" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M74" s="5"/>
       <c r="N74" s="5"/>
@@ -7541,13 +7541,13 @@
         <v>623</v>
       </c>
       <c r="J75" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="K75" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="L75" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M75" s="3"/>
       <c r="N75" s="3"/>
@@ -7581,13 +7581,13 @@
         <v>629</v>
       </c>
       <c r="J76" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K76" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L76" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M76" s="5"/>
       <c r="N76" s="5"/>
@@ -7621,13 +7621,13 @@
         <v>636</v>
       </c>
       <c r="J77" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K77" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L77" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M77" s="3"/>
       <c r="N77" s="3"/>
@@ -7661,13 +7661,13 @@
         <v>643</v>
       </c>
       <c r="J78" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K78" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L78" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M78" s="5"/>
       <c r="N78" s="5"/>
@@ -7701,13 +7701,13 @@
         <v>650</v>
       </c>
       <c r="J79" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K79" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L79" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M79" s="3"/>
       <c r="N79" s="3"/>
@@ -7741,13 +7741,13 @@
         <v>657</v>
       </c>
       <c r="J80" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K80" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L80" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M80" s="5"/>
       <c r="N80" s="5"/>
@@ -7781,13 +7781,13 @@
         <v>664</v>
       </c>
       <c r="J81" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K81" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L81" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M81" s="3"/>
       <c r="N81" s="3"/>
@@ -7821,13 +7821,13 @@
         <v>670</v>
       </c>
       <c r="J82" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K82" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L82" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M82" s="5"/>
       <c r="N82" s="5"/>
@@ -7861,13 +7861,13 @@
         <v>677</v>
       </c>
       <c r="J83" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K83" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L83" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M83" s="3"/>
       <c r="N83" s="3"/>
@@ -7901,13 +7901,13 @@
         <v>683</v>
       </c>
       <c r="J84" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K84" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L84" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M84" s="5"/>
       <c r="N84" s="5"/>
@@ -7941,13 +7941,13 @@
         <v>689</v>
       </c>
       <c r="J85" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K85" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L85" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M85" s="3"/>
       <c r="N85" s="3"/>
@@ -7981,13 +7981,13 @@
         <v>695</v>
       </c>
       <c r="J86" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K86" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L86" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M86" s="5"/>
       <c r="N86" s="5"/>
@@ -8021,13 +8021,13 @@
         <v>702</v>
       </c>
       <c r="J87" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K87" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L87" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M87" s="3"/>
       <c r="N87" s="3"/>
@@ -8061,13 +8061,13 @@
         <v>708</v>
       </c>
       <c r="J88" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K88" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L88" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M88" s="5"/>
       <c r="N88" s="5"/>
@@ -8101,13 +8101,13 @@
         <v>714</v>
       </c>
       <c r="J89" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K89" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="L89" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M89" s="3"/>
       <c r="N89" s="3"/>
@@ -8141,13 +8141,13 @@
         <v>720</v>
       </c>
       <c r="J90" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K90" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L90" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M90" s="5"/>
       <c r="N90" s="5"/>
@@ -8181,13 +8181,13 @@
         <v>726</v>
       </c>
       <c r="J91" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="K91" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="L91" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M91" s="3"/>
       <c r="N91" s="3"/>
@@ -8221,13 +8221,13 @@
         <v>732</v>
       </c>
       <c r="J92" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="K92" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="L92" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M92" s="5"/>
       <c r="N92" s="5"/>
@@ -8261,13 +8261,13 @@
         <v>738</v>
       </c>
       <c r="J93" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="K93" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="L93" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M93" s="3"/>
       <c r="N93" s="3"/>
@@ -8301,13 +8301,13 @@
         <v>744</v>
       </c>
       <c r="J94" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K94" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L94" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M94" s="5"/>
       <c r="N94" s="5"/>
@@ -8341,13 +8341,13 @@
         <v>750</v>
       </c>
       <c r="J95" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K95" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L95" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M95" s="3"/>
       <c r="N95" s="3"/>
@@ -8381,13 +8381,13 @@
         <v>757</v>
       </c>
       <c r="J96" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="K96" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="L96" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M96" s="5"/>
       <c r="N96" s="5"/>
@@ -8421,13 +8421,13 @@
         <v>764</v>
       </c>
       <c r="J97" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="K97" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="L97" s="3" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="M97" s="3"/>
       <c r="N97" s="3"/>
@@ -8461,13 +8461,13 @@
         <v>771</v>
       </c>
       <c r="J98" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K98" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L98" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M98" s="5"/>
       <c r="N98" s="5"/>
@@ -8501,13 +8501,13 @@
         <v>777</v>
       </c>
       <c r="J99" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K99" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L99" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M99" s="3"/>
       <c r="N99" s="3"/>
@@ -8541,13 +8541,13 @@
         <v>783</v>
       </c>
       <c r="J100" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K100" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L100" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M100" s="5"/>
       <c r="N100" s="5"/>
@@ -8581,13 +8581,13 @@
         <v>788</v>
       </c>
       <c r="J101" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="K101" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="L101" s="3" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M101" s="3"/>
       <c r="N101" s="3"/>
@@ -8621,13 +8621,13 @@
         <v>795</v>
       </c>
       <c r="J102" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="K102" s="5" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="L102" s="5" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="M102" s="5"/>
       <c r="N102" s="5"/>
@@ -9567,13 +9567,13 @@
         <v>8</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>1034</v>
+        <v>1031</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>1035</v>
+        <v>1032</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>1033</v>
+        <v>1030</v>
       </c>
       <c r="L2" s="6" t="s">
         <v>848</v>
@@ -9613,10 +9613,14 @@
       <c r="H3" s="3" t="s">
         <v>857</v>
       </c>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
+      <c r="I3" s="3" t="s">
+        <v>1034</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>1033</v>
+      </c>
       <c r="K3" s="2" t="s">
-        <v>1028</v>
+        <v>1038</v>
       </c>
       <c r="L3" s="3"/>
       <c r="M3" s="2"/>
@@ -9648,9 +9652,15 @@
       <c r="H4" s="5" t="s">
         <v>865</v>
       </c>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="4"/>
+      <c r="I4" s="4" t="s">
+        <v>1034</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>1034</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>1034</v>
+      </c>
       <c r="L4" s="5"/>
       <c r="M4" s="4"/>
       <c r="N4" s="5"/>
@@ -9681,9 +9691,15 @@
       <c r="H5" s="3" t="s">
         <v>873</v>
       </c>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="2"/>
+      <c r="I5" s="2" t="s">
+        <v>1034</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>1034</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>1034</v>
+      </c>
       <c r="L5" s="3"/>
       <c r="M5" s="2"/>
       <c r="N5" s="3"/>
@@ -9714,9 +9730,15 @@
       <c r="H6" s="5" t="s">
         <v>881</v>
       </c>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="4"/>
+      <c r="I6" s="4" t="s">
+        <v>1034</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>1034</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>1033</v>
+      </c>
       <c r="L6" s="5"/>
       <c r="M6" s="4"/>
       <c r="N6" s="5"/>
@@ -9747,9 +9769,15 @@
       <c r="H7" s="3" t="s">
         <v>889</v>
       </c>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="2"/>
+      <c r="I7" s="2" t="s">
+        <v>1034</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>1034</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>1034</v>
+      </c>
       <c r="L7" s="3"/>
       <c r="M7" s="2"/>
       <c r="N7" s="3"/>
@@ -9780,9 +9808,15 @@
       <c r="H8" s="5" t="s">
         <v>897</v>
       </c>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="4"/>
+      <c r="I8" s="4" t="s">
+        <v>1034</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>1034</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>1033</v>
+      </c>
       <c r="L8" s="5"/>
       <c r="M8" s="4"/>
       <c r="N8" s="5"/>
@@ -9813,9 +9847,15 @@
       <c r="H9" s="3" t="s">
         <v>905</v>
       </c>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="2"/>
+      <c r="I9" s="2" t="s">
+        <v>1034</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>1034</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>1034</v>
+      </c>
       <c r="L9" s="3"/>
       <c r="M9" s="2"/>
       <c r="N9" s="3"/>
@@ -9846,9 +9886,15 @@
       <c r="H10" s="5" t="s">
         <v>913</v>
       </c>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="4"/>
+      <c r="I10" s="4" t="s">
+        <v>1034</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>1033</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>1033</v>
+      </c>
       <c r="L10" s="5"/>
       <c r="M10" s="4"/>
       <c r="N10" s="5"/>
@@ -9879,9 +9925,15 @@
       <c r="H11" s="3" t="s">
         <v>921</v>
       </c>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="2"/>
+      <c r="I11" s="2" t="s">
+        <v>1034</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>1034</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>1034</v>
+      </c>
       <c r="L11" s="3"/>
       <c r="M11" s="2"/>
       <c r="N11" s="3"/>
@@ -9912,9 +9964,15 @@
       <c r="H12" s="5" t="s">
         <v>929</v>
       </c>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="4"/>
+      <c r="I12" s="4" t="s">
+        <v>1038</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>1033</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>1034</v>
+      </c>
       <c r="L12" s="5"/>
       <c r="M12" s="4"/>
       <c r="N12" s="5"/>
@@ -9945,9 +10003,15 @@
       <c r="H13" s="2" t="s">
         <v>937</v>
       </c>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
+      <c r="I13" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>1033</v>
+      </c>
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
       <c r="N13" s="2"/>
@@ -9978,9 +10042,15 @@
       <c r="H14" s="4" t="s">
         <v>945</v>
       </c>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
+      <c r="I14" s="4" t="s">
+        <v>1034</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>1034</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>1034</v>
+      </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4"/>
       <c r="N14" s="4"/>
@@ -10011,9 +10081,15 @@
       <c r="H15" s="2" t="s">
         <v>952</v>
       </c>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
+      <c r="I15" s="2" t="s">
+        <v>1034</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>1034</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>1034</v>
+      </c>
       <c r="L15" s="2"/>
       <c r="M15" s="2"/>
       <c r="N15" s="2"/>
@@ -10044,9 +10120,15 @@
       <c r="H16" s="4" t="s">
         <v>960</v>
       </c>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4"/>
-      <c r="K16" s="4"/>
+      <c r="I16" s="4" t="s">
+        <v>1033</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>1033</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>1033</v>
+      </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4"/>
       <c r="N16" s="4"/>
@@ -10077,9 +10159,15 @@
       <c r="H17" s="2" t="s">
         <v>967</v>
       </c>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
+      <c r="I17" s="2" t="s">
+        <v>1039</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>1034</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>1033</v>
+      </c>
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
       <c r="N17" s="2"/>
@@ -10110,9 +10198,15 @@
       <c r="H18" s="4" t="s">
         <v>975</v>
       </c>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
+      <c r="I18" s="4" t="s">
+        <v>1034</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>1033</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>1033</v>
+      </c>
       <c r="L18" s="4"/>
       <c r="M18" s="4"/>
       <c r="N18" s="4"/>
@@ -10143,9 +10237,15 @@
       <c r="H19" s="2" t="s">
         <v>982</v>
       </c>
-      <c r="I19" s="2"/>
-      <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
+      <c r="I19" s="2" t="s">
+        <v>1034</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>1034</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>1034</v>
+      </c>
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
       <c r="N19" s="2"/>
@@ -10176,9 +10276,15 @@
       <c r="H20" s="4" t="s">
         <v>990</v>
       </c>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4"/>
-      <c r="K20" s="4"/>
+      <c r="I20" s="4" t="s">
+        <v>1034</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>1034</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>1034</v>
+      </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
       <c r="N20" s="4"/>
@@ -10209,9 +10315,15 @@
       <c r="H21" s="2" t="s">
         <v>998</v>
       </c>
-      <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
+      <c r="I21" s="2" t="s">
+        <v>1034</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>1034</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>1034</v>
+      </c>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
       <c r="N21" s="2"/>
@@ -10242,9 +10354,15 @@
       <c r="H22" s="4" t="s">
         <v>1006</v>
       </c>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4"/>
+      <c r="I22" s="4" t="s">
+        <v>1033</v>
+      </c>
+      <c r="J22" s="4" t="s">
+        <v>1034</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>1033</v>
+      </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
       <c r="N22" s="4"/>
@@ -10357,13 +10475,13 @@
         <v>21</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>1028</v>
+        <v>1034</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>1029</v>
+        <v>1034</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>791</v>
+        <v>1034</v>
       </c>
       <c r="L3" s="9"/>
       <c r="M3" s="8"/>
@@ -10393,9 +10511,15 @@
       <c r="H4" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="I4" s="8"/>
-      <c r="J4" s="8"/>
-      <c r="K4" s="8"/>
+      <c r="I4" s="8" t="s">
+        <v>1034</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>1034</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>1034</v>
+      </c>
       <c r="L4" s="9"/>
       <c r="M4" s="8"/>
     </row>
@@ -10424,9 +10548,15 @@
       <c r="H5" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
-      <c r="K5" s="8"/>
+      <c r="I5" s="8" t="s">
+        <v>1034</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>1034</v>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>1034</v>
+      </c>
       <c r="L5" s="9"/>
       <c r="M5" s="8"/>
     </row>
@@ -10455,9 +10585,15 @@
       <c r="H6" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
+      <c r="I6" s="8" t="s">
+        <v>1034</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>1034</v>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>1034</v>
+      </c>
       <c r="L6" s="9"/>
       <c r="M6" s="8"/>
     </row>
@@ -10486,9 +10622,15 @@
       <c r="H7" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
+      <c r="I7" s="8" t="s">
+        <v>1034</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>1034</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>1034</v>
+      </c>
       <c r="L7" s="9"/>
       <c r="M7" s="8"/>
     </row>
@@ -10517,9 +10659,15 @@
       <c r="H8" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
+      <c r="I8" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>1033</v>
+      </c>
       <c r="L8" s="3"/>
       <c r="M8" s="2"/>
     </row>
@@ -10548,9 +10696,15 @@
       <c r="H9" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
+      <c r="I9" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>1033</v>
+      </c>
       <c r="L9" s="3"/>
       <c r="M9" s="2"/>
     </row>
@@ -10579,9 +10733,15 @@
       <c r="H10" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
+      <c r="I10" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>1033</v>
+      </c>
       <c r="L10" s="3"/>
       <c r="M10" s="2"/>
     </row>
@@ -10610,9 +10770,15 @@
       <c r="H11" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
+      <c r="I11" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>1033</v>
+      </c>
       <c r="L11" s="3"/>
       <c r="M11" s="2"/>
     </row>
@@ -10641,9 +10807,15 @@
       <c r="H12" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
-      <c r="K12" s="8"/>
+      <c r="I12" s="8" t="s">
+        <v>1033</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>1033</v>
+      </c>
+      <c r="K12" s="8" t="s">
+        <v>1033</v>
+      </c>
       <c r="L12" s="9"/>
       <c r="M12" s="8"/>
     </row>
@@ -10672,9 +10844,15 @@
       <c r="H13" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
-      <c r="K13" s="8"/>
+      <c r="I13" s="8" t="s">
+        <v>1033</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>1033</v>
+      </c>
+      <c r="K13" s="8" t="s">
+        <v>1033</v>
+      </c>
       <c r="L13" s="9"/>
       <c r="M13" s="8"/>
     </row>
@@ -10703,9 +10881,15 @@
       <c r="H14" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="I14" s="8"/>
-      <c r="J14" s="8"/>
-      <c r="K14" s="8"/>
+      <c r="I14" s="8" t="s">
+        <v>1033</v>
+      </c>
+      <c r="J14" s="8" t="s">
+        <v>1033</v>
+      </c>
+      <c r="K14" s="8" t="s">
+        <v>1033</v>
+      </c>
       <c r="L14" s="9"/>
       <c r="M14" s="8"/>
     </row>
@@ -10734,9 +10918,15 @@
       <c r="H15" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="I15" s="8"/>
-      <c r="J15" s="8"/>
-      <c r="K15" s="8"/>
+      <c r="I15" s="8" t="s">
+        <v>1033</v>
+      </c>
+      <c r="J15" s="8" t="s">
+        <v>1033</v>
+      </c>
+      <c r="K15" s="8" t="s">
+        <v>1033</v>
+      </c>
       <c r="L15" s="9"/>
       <c r="M15" s="8"/>
     </row>
@@ -10765,9 +10955,15 @@
       <c r="H16" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
+      <c r="I16" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>1033</v>
+      </c>
       <c r="L16" s="3"/>
       <c r="M16" s="2"/>
     </row>
@@ -10796,9 +10992,15 @@
       <c r="H17" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
+      <c r="I17" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>1033</v>
+      </c>
       <c r="L17" s="3"/>
       <c r="M17" s="2"/>
     </row>
@@ -10828,13 +11030,13 @@
         <v>94</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>791</v>
+        <v>1033</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>791</v>
+        <v>1033</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>791</v>
+        <v>1033</v>
       </c>
       <c r="L18" s="3"/>
       <c r="M18" s="2"/>
@@ -10864,9 +11066,15 @@
       <c r="H19" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
-      <c r="K19" s="8"/>
+      <c r="I19" s="8" t="s">
+        <v>1033</v>
+      </c>
+      <c r="J19" s="8" t="s">
+        <v>1033</v>
+      </c>
+      <c r="K19" s="8" t="s">
+        <v>1034</v>
+      </c>
       <c r="L19" s="9"/>
       <c r="M19" s="8"/>
     </row>
@@ -10895,9 +11103,15 @@
       <c r="H20" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
-      <c r="K20" s="8"/>
+      <c r="I20" s="8" t="s">
+        <v>1033</v>
+      </c>
+      <c r="J20" s="8" t="s">
+        <v>1034</v>
+      </c>
+      <c r="K20" s="8" t="s">
+        <v>1034</v>
+      </c>
       <c r="L20" s="9"/>
       <c r="M20" s="8"/>
     </row>
@@ -10926,9 +11140,15 @@
       <c r="H21" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="I21" s="8"/>
-      <c r="J21" s="8"/>
-      <c r="K21" s="8"/>
+      <c r="I21" s="8" t="s">
+        <v>1033</v>
+      </c>
+      <c r="J21" s="8" t="s">
+        <v>1034</v>
+      </c>
+      <c r="K21" s="8" t="s">
+        <v>1034</v>
+      </c>
       <c r="L21" s="9"/>
       <c r="M21" s="8"/>
     </row>
@@ -10957,9 +11177,15 @@
       <c r="H22" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="I22" s="8"/>
-      <c r="J22" s="8"/>
-      <c r="K22" s="8"/>
+      <c r="I22" s="8" t="s">
+        <v>1033</v>
+      </c>
+      <c r="J22" s="8" t="s">
+        <v>1033</v>
+      </c>
+      <c r="K22" s="8" t="s">
+        <v>1033</v>
+      </c>
       <c r="L22" s="9"/>
       <c r="M22" s="8"/>
     </row>
@@ -10988,9 +11214,15 @@
       <c r="H23" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
+      <c r="I23" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>1033</v>
+      </c>
       <c r="L23" s="3"/>
       <c r="M23" s="2"/>
     </row>
@@ -11019,9 +11251,15 @@
       <c r="H24" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
+      <c r="I24" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>1033</v>
+      </c>
       <c r="L24" s="3"/>
       <c r="M24" s="2"/>
     </row>
@@ -11050,9 +11288,15 @@
       <c r="H25" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
+      <c r="I25" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>1033</v>
+      </c>
       <c r="L25" s="3"/>
       <c r="M25" s="2"/>
     </row>

</xml_diff>

<commit_message>
Korekcije charta i worda
</commit_message>
<xml_diff>
--- a/dataset_evaluacija_llm_sa_odgovorima.xlsx
+++ b/dataset_evaluacija_llm_sa_odgovorima.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cofi24\Desktop\Git uploads\Evaluacija-jezickih-modela\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{530084F6-1F60-4FB5-8CAA-0AC376439CC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06440D9A-1B13-40C0-8D0B-7CC1F1356CF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="615" yWindow="2175" windowWidth="15600" windowHeight="11385" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tačnost" sheetId="1" r:id="rId1"/>
@@ -4137,14 +4137,14 @@
     <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4467,7 +4467,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="30"/>
@@ -4768,7 +4768,7 @@
       <c r="M8" s="5"/>
       <c r="N8" s="5"/>
     </row>
-    <row r="9" spans="1:14" ht="216.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="191.25" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>56</v>
       </c>
@@ -5076,7 +5076,7 @@
       <c r="M16" s="5"/>
       <c r="N16" s="5"/>
     </row>
-    <row r="17" spans="1:14" ht="216.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" ht="204" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>113</v>
       </c>
@@ -5116,7 +5116,7 @@
       <c r="M17" s="3"/>
       <c r="N17" s="3"/>
     </row>
-    <row r="18" spans="1:14" ht="216.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" ht="191.25" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>120</v>
       </c>
@@ -5156,7 +5156,7 @@
       <c r="M18" s="5"/>
       <c r="N18" s="5"/>
     </row>
-    <row r="19" spans="1:14" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" ht="140.25" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>127</v>
       </c>
@@ -5834,7 +5834,7 @@
       <c r="M35" s="3"/>
       <c r="N35" s="3"/>
     </row>
-    <row r="36" spans="1:14" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" ht="408" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
         <v>241</v>
       </c>
@@ -6354,7 +6354,7 @@
       <c r="M48" s="5"/>
       <c r="N48" s="5"/>
     </row>
-    <row r="49" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>326</v>
       </c>
@@ -6554,7 +6554,7 @@
       <c r="M53" s="3"/>
       <c r="N53" s="3"/>
     </row>
-    <row r="54" spans="1:14" ht="318.75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14" ht="306" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
         <v>360</v>
       </c>
@@ -6594,7 +6594,7 @@
       <c r="M54" s="5"/>
       <c r="N54" s="5"/>
     </row>
-    <row r="55" spans="1:14" ht="267.75" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14" ht="255" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>366</v>
       </c>
@@ -6634,7 +6634,7 @@
       <c r="M55" s="3"/>
       <c r="N55" s="3"/>
     </row>
-    <row r="56" spans="1:14" ht="357" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" ht="344.25" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
         <v>373</v>
       </c>
@@ -9403,7 +9403,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="32" t="s">
         <v>718</v>
       </c>
       <c r="B1" s="30"/>
@@ -10272,7 +10272,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="29" t="s">
         <v>884</v>
       </c>
       <c r="B1" s="30"/>
@@ -10440,7 +10440,7 @@
       <c r="L5" s="9"/>
       <c r="M5" s="8"/>
     </row>
-    <row r="6" spans="1:13" ht="127.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>891</v>
       </c>
@@ -10810,7 +10810,7 @@
       <c r="L15" s="9"/>
       <c r="M15" s="8"/>
     </row>
-    <row r="16" spans="1:13" ht="140.25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" ht="127.5" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>952</v>
       </c>
@@ -10921,7 +10921,7 @@
       <c r="L18" s="3"/>
       <c r="M18" s="2"/>
     </row>
-    <row r="19" spans="1:13" ht="127.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
         <v>967</v>
       </c>
@@ -11143,7 +11143,7 @@
       <c r="L24" s="3"/>
       <c r="M24" s="2"/>
     </row>
-    <row r="25" spans="1:13" ht="178.5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" ht="165.75" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>981</v>
       </c>

</xml_diff>